<commit_message>
Pre-fill agent roster and owner email in score card
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hekr7PJ49dGvUHrTGM3jGu
</commit_message>
<xml_diff>
--- a/scorecard/Praedium_Agent_Score_Card.xlsx
+++ b/scorecard/Praedium_Agent_Score_Card.xlsx
@@ -10,16 +10,16 @@
     <sheet name="Start Here" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Settings" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Agent 1 Scorecard" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Agent 1 Assessment" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Agent 2 Scorecard" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Agent 2 Assessment" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Agent 3 Scorecard" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Agent 3 Assessment" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Agent 4 Scorecard" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Agent 4 Assessment" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Agent 5 Scorecard" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Agent 5 Assessment" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Gabrielle Gillie Scorecard" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gabrielle Gillie Assessment" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Dillon Scorecard" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Dillon Assessment" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Marcus Lominick Scorecard" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Marcus Lominick Assessment" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Mary Elizabeth Young Scorecard" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Mary Elizabeth Young Assessment" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Jayan Abraham Scorecard" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Jayan Abraham Assessment" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="Agent 6 Scorecard" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="Agent 6 Assessment" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="Agent 7 Scorecard" sheetId="16" state="visible" r:id="rId16"/>
@@ -1071,7 +1071,7 @@
       </c>
       <c r="B6" s="34" t="n"/>
       <c r="C6" s="12">
-        <f>IF('Agent 4 Assessment'!C285="","",'Agent 4 Assessment'!C285)</f>
+        <f>IF('Mary Elizabeth Young Assessment'!C285="","",'Mary Elizabeth Young Assessment'!C285)</f>
         <v/>
       </c>
       <c r="D6" s="12">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="B7" s="34" t="n"/>
       <c r="C7" s="12">
-        <f>IF('Agent 4 Assessment'!C284="","",'Agent 4 Assessment'!C284)</f>
+        <f>IF('Mary Elizabeth Young Assessment'!C284="","",'Mary Elizabeth Young Assessment'!C284)</f>
         <v/>
       </c>
       <c r="D7" s="12">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="B8" s="34" t="n"/>
       <c r="C8" s="11">
-        <f>IF('Agent 4 Assessment'!C286="","",'Agent 4 Assessment'!C286)</f>
+        <f>IF('Mary Elizabeth Young Assessment'!C286="","",'Mary Elizabeth Young Assessment'!C286)</f>
         <v/>
       </c>
       <c r="D8" s="11">
@@ -1170,7 +1170,7 @@
       </c>
       <c r="B9" s="34" t="n"/>
       <c r="C9" s="11">
-        <f>IF('Agent 4 Assessment'!C287="","",'Agent 4 Assessment'!C287)</f>
+        <f>IF('Mary Elizabeth Young Assessment'!C287="","",'Mary Elizabeth Young Assessment'!C287)</f>
         <v/>
       </c>
       <c r="D9" s="11">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="B10" s="34" t="n"/>
       <c r="C10" s="11">
-        <f>IF('Agent 4 Assessment'!C288="","",'Agent 4 Assessment'!C288)</f>
+        <f>IF('Mary Elizabeth Young Assessment'!C288="","",'Mary Elizabeth Young Assessment'!C288)</f>
         <v/>
       </c>
       <c r="D10" s="11">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="B11" s="34" t="n"/>
       <c r="C11" s="11">
-        <f>IF('Agent 4 Assessment'!C289="","",'Agent 4 Assessment'!C289)</f>
+        <f>IF('Mary Elizabeth Young Assessment'!C289="","",'Mary Elizabeth Young Assessment'!C289)</f>
         <v/>
       </c>
       <c r="D11" s="11">
@@ -1257,7 +1257,7 @@
         </is>
       </c>
       <c r="K11" s="17">
-        <f>'Agent 4 Assessment'!C3</f>
+        <f>'Mary Elizabeth Young Assessment'!C3</f>
         <v/>
       </c>
     </row>
@@ -1269,7 +1269,7 @@
       </c>
       <c r="B12" s="34" t="n"/>
       <c r="C12" s="11">
-        <f>IF('Agent 4 Assessment'!C290="","",'Agent 4 Assessment'!C290*3)</f>
+        <f>IF('Mary Elizabeth Young Assessment'!C290="","",'Mary Elizabeth Young Assessment'!C290*3)</f>
         <v/>
       </c>
       <c r="D12" s="11">
@@ -7217,7 +7217,7 @@
       </c>
       <c r="B6" s="34" t="n"/>
       <c r="C6" s="12">
-        <f>IF('Agent 5 Assessment'!C285="","",'Agent 5 Assessment'!C285)</f>
+        <f>IF('Jayan Abraham Assessment'!C285="","",'Jayan Abraham Assessment'!C285)</f>
         <v/>
       </c>
       <c r="D6" s="12">
@@ -7250,7 +7250,7 @@
       </c>
       <c r="B7" s="34" t="n"/>
       <c r="C7" s="12">
-        <f>IF('Agent 5 Assessment'!C284="","",'Agent 5 Assessment'!C284)</f>
+        <f>IF('Jayan Abraham Assessment'!C284="","",'Jayan Abraham Assessment'!C284)</f>
         <v/>
       </c>
       <c r="D7" s="12">
@@ -7283,7 +7283,7 @@
       </c>
       <c r="B8" s="34" t="n"/>
       <c r="C8" s="11">
-        <f>IF('Agent 5 Assessment'!C286="","",'Agent 5 Assessment'!C286)</f>
+        <f>IF('Jayan Abraham Assessment'!C286="","",'Jayan Abraham Assessment'!C286)</f>
         <v/>
       </c>
       <c r="D8" s="11">
@@ -7316,7 +7316,7 @@
       </c>
       <c r="B9" s="34" t="n"/>
       <c r="C9" s="11">
-        <f>IF('Agent 5 Assessment'!C287="","",'Agent 5 Assessment'!C287)</f>
+        <f>IF('Jayan Abraham Assessment'!C287="","",'Jayan Abraham Assessment'!C287)</f>
         <v/>
       </c>
       <c r="D9" s="11">
@@ -7349,7 +7349,7 @@
       </c>
       <c r="B10" s="34" t="n"/>
       <c r="C10" s="11">
-        <f>IF('Agent 5 Assessment'!C288="","",'Agent 5 Assessment'!C288)</f>
+        <f>IF('Jayan Abraham Assessment'!C288="","",'Jayan Abraham Assessment'!C288)</f>
         <v/>
       </c>
       <c r="D10" s="11">
@@ -7382,7 +7382,7 @@
       </c>
       <c r="B11" s="34" t="n"/>
       <c r="C11" s="11">
-        <f>IF('Agent 5 Assessment'!C289="","",'Agent 5 Assessment'!C289)</f>
+        <f>IF('Jayan Abraham Assessment'!C289="","",'Jayan Abraham Assessment'!C289)</f>
         <v/>
       </c>
       <c r="D11" s="11">
@@ -7403,7 +7403,7 @@
         </is>
       </c>
       <c r="K11" s="17">
-        <f>'Agent 5 Assessment'!C3</f>
+        <f>'Jayan Abraham Assessment'!C3</f>
         <v/>
       </c>
     </row>
@@ -7415,7 +7415,7 @@
       </c>
       <c r="B12" s="34" t="n"/>
       <c r="C12" s="11">
-        <f>IF('Agent 5 Assessment'!C290="","",'Agent 5 Assessment'!C290*3)</f>
+        <f>IF('Jayan Abraham Assessment'!C290="","",'Jayan Abraham Assessment'!C290*3)</f>
         <v/>
       </c>
       <c r="D12" s="11">
@@ -25735,91 +25735,91 @@
         <v/>
       </c>
       <c r="B6" s="10">
-        <f>'Agent 1 Assessment'!C3</f>
+        <f>'Gabrielle Gillie Assessment'!C3</f>
         <v/>
       </c>
       <c r="C6" s="11">
-        <f>IFERROR(INDEX('Agent 1 Scorecard'!$Z$15:$Z$80,MATCH($B$3,'Agent 1 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Gabrielle Gillie Scorecard'!$Z$15:$Z$80,MATCH($B$3,'Gabrielle Gillie Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>IFERROR(INDEX('Agent 1 Scorecard'!$C$15:$C$80,MATCH($B$3,'Agent 1 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Gabrielle Gillie Scorecard'!$C$15:$C$80,MATCH($B$3,'Gabrielle Gillie Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="E6" s="11">
-        <f>IFERROR(INDEX('Agent 1 Scorecard'!$E$15:$E$80,MATCH($B$3,'Agent 1 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Gabrielle Gillie Scorecard'!$E$15:$E$80,MATCH($B$3,'Gabrielle Gillie Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="F6" s="11">
-        <f>IFERROR(INDEX('Agent 1 Scorecard'!$F$15:$F$80,MATCH($B$3,'Agent 1 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Gabrielle Gillie Scorecard'!$F$15:$F$80,MATCH($B$3,'Gabrielle Gillie Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="G6" s="11">
-        <f>IFERROR(INDEX('Agent 1 Scorecard'!$G$15:$G$80,MATCH($B$3,'Agent 1 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Gabrielle Gillie Scorecard'!$G$15:$G$80,MATCH($B$3,'Gabrielle Gillie Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="H6" s="11">
-        <f>IFERROR(INDEX('Agent 1 Scorecard'!$H$15:$H$80,MATCH($B$3,'Agent 1 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Gabrielle Gillie Scorecard'!$H$15:$H$80,MATCH($B$3,'Gabrielle Gillie Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="I6" s="11">
-        <f>IFERROR(INDEX('Agent 1 Scorecard'!$I$15:$I$80,MATCH($B$3,'Agent 1 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Gabrielle Gillie Scorecard'!$I$15:$I$80,MATCH($B$3,'Gabrielle Gillie Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="J6" s="11">
-        <f>IFERROR(INDEX('Agent 1 Scorecard'!$J$15:$J$80,MATCH($B$3,'Agent 1 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Gabrielle Gillie Scorecard'!$J$15:$J$80,MATCH($B$3,'Gabrielle Gillie Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="K6" s="11">
-        <f>IFERROR(INDEX('Agent 1 Scorecard'!$K$15:$K$80,MATCH($B$3,'Agent 1 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Gabrielle Gillie Scorecard'!$K$15:$K$80,MATCH($B$3,'Gabrielle Gillie Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="L6" s="11">
-        <f>IFERROR(INDEX('Agent 1 Scorecard'!$L$15:$L$80,MATCH($B$3,'Agent 1 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Gabrielle Gillie Scorecard'!$L$15:$L$80,MATCH($B$3,'Gabrielle Gillie Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="M6" s="12">
-        <f>'Agent 1 Scorecard'!K10</f>
+        <f>'Gabrielle Gillie Scorecard'!K10</f>
         <v/>
       </c>
       <c r="N6" s="12">
-        <f>'Agent 1 Scorecard'!D6</f>
+        <f>'Gabrielle Gillie Scorecard'!D6</f>
         <v/>
       </c>
       <c r="O6" s="12">
-        <f>'Agent 1 Scorecard'!C6</f>
+        <f>'Gabrielle Gillie Scorecard'!C6</f>
         <v/>
       </c>
       <c r="P6" s="10">
-        <f>'Agent 1 Scorecard'!E6</f>
+        <f>'Gabrielle Gillie Scorecard'!E6</f>
         <v/>
       </c>
       <c r="Q6" s="11">
-        <f>'Agent 1 Scorecard'!D8</f>
+        <f>'Gabrielle Gillie Scorecard'!D8</f>
         <v/>
       </c>
       <c r="R6" s="11">
-        <f>'Agent 1 Scorecard'!C8</f>
+        <f>'Gabrielle Gillie Scorecard'!C8</f>
         <v/>
       </c>
       <c r="S6" s="10">
-        <f>'Agent 1 Scorecard'!K7</f>
+        <f>'Gabrielle Gillie Scorecard'!K7</f>
         <v/>
       </c>
       <c r="T6" s="13">
-        <f>'Agent 1 Scorecard'!K8</f>
+        <f>'Gabrielle Gillie Scorecard'!K8</f>
         <v/>
       </c>
       <c r="U6" s="14">
-        <f>IF(MAX('Agent 1 Scorecard'!$Y$15:$Y$80)=0,"",MAX('Agent 1 Scorecard'!$Y$15:$Y$80))</f>
+        <f>IF(MAX('Gabrielle Gillie Scorecard'!$Y$15:$Y$80)=0,"",MAX('Gabrielle Gillie Scorecard'!$Y$15:$Y$80))</f>
         <v/>
       </c>
       <c r="V6" s="15">
-        <f>IFERROR(INDEX('Agent 1 Scorecard'!$V$15:$V$80,MATCH($B$3,'Agent 1 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Gabrielle Gillie Scorecard'!$V$15:$V$80,MATCH($B$3,'Gabrielle Gillie Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="W6" s="15">
-        <f>IFERROR(INDEX('Agent 1 Scorecard'!$W$15:$W$80,MATCH($B$3,'Agent 1 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Gabrielle Gillie Scorecard'!$W$15:$W$80,MATCH($B$3,'Gabrielle Gillie Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -25829,91 +25829,91 @@
         <v/>
       </c>
       <c r="B7" s="17">
-        <f>'Agent 2 Assessment'!C3</f>
+        <f>'Dillon Assessment'!C3</f>
         <v/>
       </c>
       <c r="C7" s="18">
-        <f>IFERROR(INDEX('Agent 2 Scorecard'!$Z$15:$Z$80,MATCH($B$3,'Agent 2 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Dillon Scorecard'!$Z$15:$Z$80,MATCH($B$3,'Dillon Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="D7" s="18">
-        <f>IFERROR(INDEX('Agent 2 Scorecard'!$C$15:$C$80,MATCH($B$3,'Agent 2 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Dillon Scorecard'!$C$15:$C$80,MATCH($B$3,'Dillon Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="E7" s="18">
-        <f>IFERROR(INDEX('Agent 2 Scorecard'!$E$15:$E$80,MATCH($B$3,'Agent 2 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Dillon Scorecard'!$E$15:$E$80,MATCH($B$3,'Dillon Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="F7" s="18">
-        <f>IFERROR(INDEX('Agent 2 Scorecard'!$F$15:$F$80,MATCH($B$3,'Agent 2 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Dillon Scorecard'!$F$15:$F$80,MATCH($B$3,'Dillon Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="G7" s="18">
-        <f>IFERROR(INDEX('Agent 2 Scorecard'!$G$15:$G$80,MATCH($B$3,'Agent 2 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Dillon Scorecard'!$G$15:$G$80,MATCH($B$3,'Dillon Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="H7" s="18">
-        <f>IFERROR(INDEX('Agent 2 Scorecard'!$H$15:$H$80,MATCH($B$3,'Agent 2 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Dillon Scorecard'!$H$15:$H$80,MATCH($B$3,'Dillon Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="I7" s="18">
-        <f>IFERROR(INDEX('Agent 2 Scorecard'!$I$15:$I$80,MATCH($B$3,'Agent 2 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Dillon Scorecard'!$I$15:$I$80,MATCH($B$3,'Dillon Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="J7" s="18">
-        <f>IFERROR(INDEX('Agent 2 Scorecard'!$J$15:$J$80,MATCH($B$3,'Agent 2 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Dillon Scorecard'!$J$15:$J$80,MATCH($B$3,'Dillon Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="K7" s="18">
-        <f>IFERROR(INDEX('Agent 2 Scorecard'!$K$15:$K$80,MATCH($B$3,'Agent 2 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Dillon Scorecard'!$K$15:$K$80,MATCH($B$3,'Dillon Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>IFERROR(INDEX('Agent 2 Scorecard'!$L$15:$L$80,MATCH($B$3,'Agent 2 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Dillon Scorecard'!$L$15:$L$80,MATCH($B$3,'Dillon Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="M7" s="19">
-        <f>'Agent 2 Scorecard'!K10</f>
+        <f>'Dillon Scorecard'!K10</f>
         <v/>
       </c>
       <c r="N7" s="19">
-        <f>'Agent 2 Scorecard'!D6</f>
+        <f>'Dillon Scorecard'!D6</f>
         <v/>
       </c>
       <c r="O7" s="19">
-        <f>'Agent 2 Scorecard'!C6</f>
+        <f>'Dillon Scorecard'!C6</f>
         <v/>
       </c>
       <c r="P7" s="17">
-        <f>'Agent 2 Scorecard'!E6</f>
+        <f>'Dillon Scorecard'!E6</f>
         <v/>
       </c>
       <c r="Q7" s="18">
-        <f>'Agent 2 Scorecard'!D8</f>
+        <f>'Dillon Scorecard'!D8</f>
         <v/>
       </c>
       <c r="R7" s="18">
-        <f>'Agent 2 Scorecard'!C8</f>
+        <f>'Dillon Scorecard'!C8</f>
         <v/>
       </c>
       <c r="S7" s="17">
-        <f>'Agent 2 Scorecard'!K7</f>
+        <f>'Dillon Scorecard'!K7</f>
         <v/>
       </c>
       <c r="T7" s="20">
-        <f>'Agent 2 Scorecard'!K8</f>
+        <f>'Dillon Scorecard'!K8</f>
         <v/>
       </c>
       <c r="U7" s="21">
-        <f>IF(MAX('Agent 2 Scorecard'!$Y$15:$Y$80)=0,"",MAX('Agent 2 Scorecard'!$Y$15:$Y$80))</f>
+        <f>IF(MAX('Dillon Scorecard'!$Y$15:$Y$80)=0,"",MAX('Dillon Scorecard'!$Y$15:$Y$80))</f>
         <v/>
       </c>
       <c r="V7" s="22">
-        <f>IFERROR(INDEX('Agent 2 Scorecard'!$V$15:$V$80,MATCH($B$3,'Agent 2 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Dillon Scorecard'!$V$15:$V$80,MATCH($B$3,'Dillon Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="W7" s="22">
-        <f>IFERROR(INDEX('Agent 2 Scorecard'!$W$15:$W$80,MATCH($B$3,'Agent 2 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Dillon Scorecard'!$W$15:$W$80,MATCH($B$3,'Dillon Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -25923,91 +25923,91 @@
         <v/>
       </c>
       <c r="B8" s="10">
-        <f>'Agent 3 Assessment'!C3</f>
+        <f>'Marcus Lominick Assessment'!C3</f>
         <v/>
       </c>
       <c r="C8" s="11">
-        <f>IFERROR(INDEX('Agent 3 Scorecard'!$Z$15:$Z$80,MATCH($B$3,'Agent 3 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Marcus Lominick Scorecard'!$Z$15:$Z$80,MATCH($B$3,'Marcus Lominick Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="D8" s="11">
-        <f>IFERROR(INDEX('Agent 3 Scorecard'!$C$15:$C$80,MATCH($B$3,'Agent 3 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Marcus Lominick Scorecard'!$C$15:$C$80,MATCH($B$3,'Marcus Lominick Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="E8" s="11">
-        <f>IFERROR(INDEX('Agent 3 Scorecard'!$E$15:$E$80,MATCH($B$3,'Agent 3 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Marcus Lominick Scorecard'!$E$15:$E$80,MATCH($B$3,'Marcus Lominick Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="F8" s="11">
-        <f>IFERROR(INDEX('Agent 3 Scorecard'!$F$15:$F$80,MATCH($B$3,'Agent 3 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Marcus Lominick Scorecard'!$F$15:$F$80,MATCH($B$3,'Marcus Lominick Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="G8" s="11">
-        <f>IFERROR(INDEX('Agent 3 Scorecard'!$G$15:$G$80,MATCH($B$3,'Agent 3 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Marcus Lominick Scorecard'!$G$15:$G$80,MATCH($B$3,'Marcus Lominick Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="H8" s="11">
-        <f>IFERROR(INDEX('Agent 3 Scorecard'!$H$15:$H$80,MATCH($B$3,'Agent 3 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Marcus Lominick Scorecard'!$H$15:$H$80,MATCH($B$3,'Marcus Lominick Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="I8" s="11">
-        <f>IFERROR(INDEX('Agent 3 Scorecard'!$I$15:$I$80,MATCH($B$3,'Agent 3 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Marcus Lominick Scorecard'!$I$15:$I$80,MATCH($B$3,'Marcus Lominick Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="J8" s="11">
-        <f>IFERROR(INDEX('Agent 3 Scorecard'!$J$15:$J$80,MATCH($B$3,'Agent 3 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Marcus Lominick Scorecard'!$J$15:$J$80,MATCH($B$3,'Marcus Lominick Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="K8" s="11">
-        <f>IFERROR(INDEX('Agent 3 Scorecard'!$K$15:$K$80,MATCH($B$3,'Agent 3 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Marcus Lominick Scorecard'!$K$15:$K$80,MATCH($B$3,'Marcus Lominick Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="L8" s="11">
-        <f>IFERROR(INDEX('Agent 3 Scorecard'!$L$15:$L$80,MATCH($B$3,'Agent 3 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Marcus Lominick Scorecard'!$L$15:$L$80,MATCH($B$3,'Marcus Lominick Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="M8" s="12">
-        <f>'Agent 3 Scorecard'!K10</f>
+        <f>'Marcus Lominick Scorecard'!K10</f>
         <v/>
       </c>
       <c r="N8" s="12">
-        <f>'Agent 3 Scorecard'!D6</f>
+        <f>'Marcus Lominick Scorecard'!D6</f>
         <v/>
       </c>
       <c r="O8" s="12">
-        <f>'Agent 3 Scorecard'!C6</f>
+        <f>'Marcus Lominick Scorecard'!C6</f>
         <v/>
       </c>
       <c r="P8" s="10">
-        <f>'Agent 3 Scorecard'!E6</f>
+        <f>'Marcus Lominick Scorecard'!E6</f>
         <v/>
       </c>
       <c r="Q8" s="11">
-        <f>'Agent 3 Scorecard'!D8</f>
+        <f>'Marcus Lominick Scorecard'!D8</f>
         <v/>
       </c>
       <c r="R8" s="11">
-        <f>'Agent 3 Scorecard'!C8</f>
+        <f>'Marcus Lominick Scorecard'!C8</f>
         <v/>
       </c>
       <c r="S8" s="10">
-        <f>'Agent 3 Scorecard'!K7</f>
+        <f>'Marcus Lominick Scorecard'!K7</f>
         <v/>
       </c>
       <c r="T8" s="13">
-        <f>'Agent 3 Scorecard'!K8</f>
+        <f>'Marcus Lominick Scorecard'!K8</f>
         <v/>
       </c>
       <c r="U8" s="14">
-        <f>IF(MAX('Agent 3 Scorecard'!$Y$15:$Y$80)=0,"",MAX('Agent 3 Scorecard'!$Y$15:$Y$80))</f>
+        <f>IF(MAX('Marcus Lominick Scorecard'!$Y$15:$Y$80)=0,"",MAX('Marcus Lominick Scorecard'!$Y$15:$Y$80))</f>
         <v/>
       </c>
       <c r="V8" s="15">
-        <f>IFERROR(INDEX('Agent 3 Scorecard'!$V$15:$V$80,MATCH($B$3,'Agent 3 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Marcus Lominick Scorecard'!$V$15:$V$80,MATCH($B$3,'Marcus Lominick Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="W8" s="15">
-        <f>IFERROR(INDEX('Agent 3 Scorecard'!$W$15:$W$80,MATCH($B$3,'Agent 3 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Marcus Lominick Scorecard'!$W$15:$W$80,MATCH($B$3,'Marcus Lominick Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -26017,91 +26017,91 @@
         <v/>
       </c>
       <c r="B9" s="17">
-        <f>'Agent 4 Assessment'!C3</f>
+        <f>'Mary Elizabeth Young Assessment'!C3</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>IFERROR(INDEX('Agent 4 Scorecard'!$Z$15:$Z$80,MATCH($B$3,'Agent 4 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Mary Elizabeth Young Scorecard'!$Z$15:$Z$80,MATCH($B$3,'Mary Elizabeth Young Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="D9" s="18">
-        <f>IFERROR(INDEX('Agent 4 Scorecard'!$C$15:$C$80,MATCH($B$3,'Agent 4 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Mary Elizabeth Young Scorecard'!$C$15:$C$80,MATCH($B$3,'Mary Elizabeth Young Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="E9" s="18">
-        <f>IFERROR(INDEX('Agent 4 Scorecard'!$E$15:$E$80,MATCH($B$3,'Agent 4 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Mary Elizabeth Young Scorecard'!$E$15:$E$80,MATCH($B$3,'Mary Elizabeth Young Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="F9" s="18">
-        <f>IFERROR(INDEX('Agent 4 Scorecard'!$F$15:$F$80,MATCH($B$3,'Agent 4 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Mary Elizabeth Young Scorecard'!$F$15:$F$80,MATCH($B$3,'Mary Elizabeth Young Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="G9" s="18">
-        <f>IFERROR(INDEX('Agent 4 Scorecard'!$G$15:$G$80,MATCH($B$3,'Agent 4 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Mary Elizabeth Young Scorecard'!$G$15:$G$80,MATCH($B$3,'Mary Elizabeth Young Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="H9" s="18">
-        <f>IFERROR(INDEX('Agent 4 Scorecard'!$H$15:$H$80,MATCH($B$3,'Agent 4 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Mary Elizabeth Young Scorecard'!$H$15:$H$80,MATCH($B$3,'Mary Elizabeth Young Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="I9" s="18">
-        <f>IFERROR(INDEX('Agent 4 Scorecard'!$I$15:$I$80,MATCH($B$3,'Agent 4 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Mary Elizabeth Young Scorecard'!$I$15:$I$80,MATCH($B$3,'Mary Elizabeth Young Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="J9" s="18">
-        <f>IFERROR(INDEX('Agent 4 Scorecard'!$J$15:$J$80,MATCH($B$3,'Agent 4 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Mary Elizabeth Young Scorecard'!$J$15:$J$80,MATCH($B$3,'Mary Elizabeth Young Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="K9" s="18">
-        <f>IFERROR(INDEX('Agent 4 Scorecard'!$K$15:$K$80,MATCH($B$3,'Agent 4 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Mary Elizabeth Young Scorecard'!$K$15:$K$80,MATCH($B$3,'Mary Elizabeth Young Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>IFERROR(INDEX('Agent 4 Scorecard'!$L$15:$L$80,MATCH($B$3,'Agent 4 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Mary Elizabeth Young Scorecard'!$L$15:$L$80,MATCH($B$3,'Mary Elizabeth Young Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="M9" s="19">
-        <f>'Agent 4 Scorecard'!K10</f>
+        <f>'Mary Elizabeth Young Scorecard'!K10</f>
         <v/>
       </c>
       <c r="N9" s="19">
-        <f>'Agent 4 Scorecard'!D6</f>
+        <f>'Mary Elizabeth Young Scorecard'!D6</f>
         <v/>
       </c>
       <c r="O9" s="19">
-        <f>'Agent 4 Scorecard'!C6</f>
+        <f>'Mary Elizabeth Young Scorecard'!C6</f>
         <v/>
       </c>
       <c r="P9" s="17">
-        <f>'Agent 4 Scorecard'!E6</f>
+        <f>'Mary Elizabeth Young Scorecard'!E6</f>
         <v/>
       </c>
       <c r="Q9" s="18">
-        <f>'Agent 4 Scorecard'!D8</f>
+        <f>'Mary Elizabeth Young Scorecard'!D8</f>
         <v/>
       </c>
       <c r="R9" s="18">
-        <f>'Agent 4 Scorecard'!C8</f>
+        <f>'Mary Elizabeth Young Scorecard'!C8</f>
         <v/>
       </c>
       <c r="S9" s="17">
-        <f>'Agent 4 Scorecard'!K7</f>
+        <f>'Mary Elizabeth Young Scorecard'!K7</f>
         <v/>
       </c>
       <c r="T9" s="20">
-        <f>'Agent 4 Scorecard'!K8</f>
+        <f>'Mary Elizabeth Young Scorecard'!K8</f>
         <v/>
       </c>
       <c r="U9" s="21">
-        <f>IF(MAX('Agent 4 Scorecard'!$Y$15:$Y$80)=0,"",MAX('Agent 4 Scorecard'!$Y$15:$Y$80))</f>
+        <f>IF(MAX('Mary Elizabeth Young Scorecard'!$Y$15:$Y$80)=0,"",MAX('Mary Elizabeth Young Scorecard'!$Y$15:$Y$80))</f>
         <v/>
       </c>
       <c r="V9" s="22">
-        <f>IFERROR(INDEX('Agent 4 Scorecard'!$V$15:$V$80,MATCH($B$3,'Agent 4 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Mary Elizabeth Young Scorecard'!$V$15:$V$80,MATCH($B$3,'Mary Elizabeth Young Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="W9" s="22">
-        <f>IFERROR(INDEX('Agent 4 Scorecard'!$W$15:$W$80,MATCH($B$3,'Agent 4 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Mary Elizabeth Young Scorecard'!$W$15:$W$80,MATCH($B$3,'Mary Elizabeth Young Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -26111,91 +26111,91 @@
         <v/>
       </c>
       <c r="B10" s="10">
-        <f>'Agent 5 Assessment'!C3</f>
+        <f>'Jayan Abraham Assessment'!C3</f>
         <v/>
       </c>
       <c r="C10" s="11">
-        <f>IFERROR(INDEX('Agent 5 Scorecard'!$Z$15:$Z$80,MATCH($B$3,'Agent 5 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Jayan Abraham Scorecard'!$Z$15:$Z$80,MATCH($B$3,'Jayan Abraham Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="D10" s="11">
-        <f>IFERROR(INDEX('Agent 5 Scorecard'!$C$15:$C$80,MATCH($B$3,'Agent 5 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Jayan Abraham Scorecard'!$C$15:$C$80,MATCH($B$3,'Jayan Abraham Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="E10" s="11">
-        <f>IFERROR(INDEX('Agent 5 Scorecard'!$E$15:$E$80,MATCH($B$3,'Agent 5 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Jayan Abraham Scorecard'!$E$15:$E$80,MATCH($B$3,'Jayan Abraham Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="F10" s="11">
-        <f>IFERROR(INDEX('Agent 5 Scorecard'!$F$15:$F$80,MATCH($B$3,'Agent 5 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Jayan Abraham Scorecard'!$F$15:$F$80,MATCH($B$3,'Jayan Abraham Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="G10" s="11">
-        <f>IFERROR(INDEX('Agent 5 Scorecard'!$G$15:$G$80,MATCH($B$3,'Agent 5 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Jayan Abraham Scorecard'!$G$15:$G$80,MATCH($B$3,'Jayan Abraham Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="H10" s="11">
-        <f>IFERROR(INDEX('Agent 5 Scorecard'!$H$15:$H$80,MATCH($B$3,'Agent 5 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Jayan Abraham Scorecard'!$H$15:$H$80,MATCH($B$3,'Jayan Abraham Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="I10" s="11">
-        <f>IFERROR(INDEX('Agent 5 Scorecard'!$I$15:$I$80,MATCH($B$3,'Agent 5 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Jayan Abraham Scorecard'!$I$15:$I$80,MATCH($B$3,'Jayan Abraham Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="J10" s="11">
-        <f>IFERROR(INDEX('Agent 5 Scorecard'!$J$15:$J$80,MATCH($B$3,'Agent 5 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Jayan Abraham Scorecard'!$J$15:$J$80,MATCH($B$3,'Jayan Abraham Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="K10" s="11">
-        <f>IFERROR(INDEX('Agent 5 Scorecard'!$K$15:$K$80,MATCH($B$3,'Agent 5 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Jayan Abraham Scorecard'!$K$15:$K$80,MATCH($B$3,'Jayan Abraham Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="L10" s="11">
-        <f>IFERROR(INDEX('Agent 5 Scorecard'!$L$15:$L$80,MATCH($B$3,'Agent 5 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Jayan Abraham Scorecard'!$L$15:$L$80,MATCH($B$3,'Jayan Abraham Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="M10" s="12">
-        <f>'Agent 5 Scorecard'!K10</f>
+        <f>'Jayan Abraham Scorecard'!K10</f>
         <v/>
       </c>
       <c r="N10" s="12">
-        <f>'Agent 5 Scorecard'!D6</f>
+        <f>'Jayan Abraham Scorecard'!D6</f>
         <v/>
       </c>
       <c r="O10" s="12">
-        <f>'Agent 5 Scorecard'!C6</f>
+        <f>'Jayan Abraham Scorecard'!C6</f>
         <v/>
       </c>
       <c r="P10" s="10">
-        <f>'Agent 5 Scorecard'!E6</f>
+        <f>'Jayan Abraham Scorecard'!E6</f>
         <v/>
       </c>
       <c r="Q10" s="11">
-        <f>'Agent 5 Scorecard'!D8</f>
+        <f>'Jayan Abraham Scorecard'!D8</f>
         <v/>
       </c>
       <c r="R10" s="11">
-        <f>'Agent 5 Scorecard'!C8</f>
+        <f>'Jayan Abraham Scorecard'!C8</f>
         <v/>
       </c>
       <c r="S10" s="10">
-        <f>'Agent 5 Scorecard'!K7</f>
+        <f>'Jayan Abraham Scorecard'!K7</f>
         <v/>
       </c>
       <c r="T10" s="13">
-        <f>'Agent 5 Scorecard'!K8</f>
+        <f>'Jayan Abraham Scorecard'!K8</f>
         <v/>
       </c>
       <c r="U10" s="14">
-        <f>IF(MAX('Agent 5 Scorecard'!$Y$15:$Y$80)=0,"",MAX('Agent 5 Scorecard'!$Y$15:$Y$80))</f>
+        <f>IF(MAX('Jayan Abraham Scorecard'!$Y$15:$Y$80)=0,"",MAX('Jayan Abraham Scorecard'!$Y$15:$Y$80))</f>
         <v/>
       </c>
       <c r="V10" s="15">
-        <f>IFERROR(INDEX('Agent 5 Scorecard'!$V$15:$V$80,MATCH($B$3,'Agent 5 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Jayan Abraham Scorecard'!$V$15:$V$80,MATCH($B$3,'Jayan Abraham Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="W10" s="15">
-        <f>IFERROR(INDEX('Agent 5 Scorecard'!$W$15:$W$80,MATCH($B$3,'Agent 5 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Jayan Abraham Scorecard'!$W$15:$W$80,MATCH($B$3,'Jayan Abraham Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -26522,7 +26522,7 @@
       </c>
       <c r="C5" s="26" t="inlineStr">
         <is>
-          <t>nicholascarnes45@gmail.com</t>
+          <t>ncarnes@kw.com</t>
         </is>
       </c>
     </row>
@@ -26630,16 +26630,24 @@
       <c r="A14" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="B14" s="28" t="inlineStr"/>
-      <c r="C14" s="28" t="inlineStr"/>
+      <c r="B14" s="28" t="inlineStr">
+        <is>
+          <t>Gabrielle Gillie</t>
+        </is>
+      </c>
+      <c r="C14" s="28" t="inlineStr">
+        <is>
+          <t>gabeg@kwcommercial.com</t>
+        </is>
+      </c>
       <c r="D14" s="29" t="inlineStr">
         <is>
-          <t>Agent 1 Scorecard</t>
+          <t>Gabrielle Gillie Scorecard</t>
         </is>
       </c>
       <c r="E14" s="29" t="inlineStr">
         <is>
-          <t>Agent 1 Assessment</t>
+          <t>Gabrielle Gillie Assessment</t>
         </is>
       </c>
       <c r="F14" s="28" t="inlineStr"/>
@@ -26648,16 +26656,24 @@
       <c r="A15" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="B15" s="28" t="inlineStr"/>
-      <c r="C15" s="28" t="inlineStr"/>
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t>Dillon</t>
+        </is>
+      </c>
+      <c r="C15" s="28" t="inlineStr">
+        <is>
+          <t>dillon2403@gmail.com</t>
+        </is>
+      </c>
       <c r="D15" s="29" t="inlineStr">
         <is>
-          <t>Agent 2 Scorecard</t>
+          <t>Dillon Scorecard</t>
         </is>
       </c>
       <c r="E15" s="29" t="inlineStr">
         <is>
-          <t>Agent 2 Assessment</t>
+          <t>Dillon Assessment</t>
         </is>
       </c>
       <c r="F15" s="28" t="inlineStr"/>
@@ -26666,16 +26682,24 @@
       <c r="A16" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="B16" s="28" t="inlineStr"/>
-      <c r="C16" s="28" t="inlineStr"/>
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>Marcus Lominick</t>
+        </is>
+      </c>
+      <c r="C16" s="28" t="inlineStr">
+        <is>
+          <t>mlominick@kwcommercial.com</t>
+        </is>
+      </c>
       <c r="D16" s="29" t="inlineStr">
         <is>
-          <t>Agent 3 Scorecard</t>
+          <t>Marcus Lominick Scorecard</t>
         </is>
       </c>
       <c r="E16" s="29" t="inlineStr">
         <is>
-          <t>Agent 3 Assessment</t>
+          <t>Marcus Lominick Assessment</t>
         </is>
       </c>
       <c r="F16" s="28" t="inlineStr"/>
@@ -26684,16 +26708,24 @@
       <c r="A17" s="27" t="n">
         <v>4</v>
       </c>
-      <c r="B17" s="28" t="inlineStr"/>
-      <c r="C17" s="28" t="inlineStr"/>
+      <c r="B17" s="28" t="inlineStr">
+        <is>
+          <t>Mary Elizabeth Young</t>
+        </is>
+      </c>
+      <c r="C17" s="28" t="inlineStr">
+        <is>
+          <t>myoung@kwcommercial.com</t>
+        </is>
+      </c>
       <c r="D17" s="29" t="inlineStr">
         <is>
-          <t>Agent 4 Scorecard</t>
+          <t>Mary Elizabeth Young Scorecard</t>
         </is>
       </c>
       <c r="E17" s="29" t="inlineStr">
         <is>
-          <t>Agent 4 Assessment</t>
+          <t>Mary Elizabeth Young Assessment</t>
         </is>
       </c>
       <c r="F17" s="28" t="inlineStr"/>
@@ -26702,16 +26734,24 @@
       <c r="A18" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="B18" s="28" t="inlineStr"/>
-      <c r="C18" s="28" t="inlineStr"/>
+      <c r="B18" s="28" t="inlineStr">
+        <is>
+          <t>Jayan Abraham</t>
+        </is>
+      </c>
+      <c r="C18" s="28" t="inlineStr">
+        <is>
+          <t>jayanabraham@kw.com</t>
+        </is>
+      </c>
       <c r="D18" s="29" t="inlineStr">
         <is>
-          <t>Agent 5 Scorecard</t>
+          <t>Jayan Abraham Scorecard</t>
         </is>
       </c>
       <c r="E18" s="29" t="inlineStr">
         <is>
-          <t>Agent 5 Assessment</t>
+          <t>Jayan Abraham Assessment</t>
         </is>
       </c>
       <c r="F18" s="28" t="inlineStr"/>
@@ -26895,7 +26935,7 @@
       </c>
       <c r="B6" s="34" t="n"/>
       <c r="C6" s="12">
-        <f>IF('Agent 1 Assessment'!C285="","",'Agent 1 Assessment'!C285)</f>
+        <f>IF('Gabrielle Gillie Assessment'!C285="","",'Gabrielle Gillie Assessment'!C285)</f>
         <v/>
       </c>
       <c r="D6" s="12">
@@ -26928,7 +26968,7 @@
       </c>
       <c r="B7" s="34" t="n"/>
       <c r="C7" s="12">
-        <f>IF('Agent 1 Assessment'!C284="","",'Agent 1 Assessment'!C284)</f>
+        <f>IF('Gabrielle Gillie Assessment'!C284="","",'Gabrielle Gillie Assessment'!C284)</f>
         <v/>
       </c>
       <c r="D7" s="12">
@@ -26961,7 +27001,7 @@
       </c>
       <c r="B8" s="34" t="n"/>
       <c r="C8" s="11">
-        <f>IF('Agent 1 Assessment'!C286="","",'Agent 1 Assessment'!C286)</f>
+        <f>IF('Gabrielle Gillie Assessment'!C286="","",'Gabrielle Gillie Assessment'!C286)</f>
         <v/>
       </c>
       <c r="D8" s="11">
@@ -26994,7 +27034,7 @@
       </c>
       <c r="B9" s="34" t="n"/>
       <c r="C9" s="11">
-        <f>IF('Agent 1 Assessment'!C287="","",'Agent 1 Assessment'!C287)</f>
+        <f>IF('Gabrielle Gillie Assessment'!C287="","",'Gabrielle Gillie Assessment'!C287)</f>
         <v/>
       </c>
       <c r="D9" s="11">
@@ -27027,7 +27067,7 @@
       </c>
       <c r="B10" s="34" t="n"/>
       <c r="C10" s="11">
-        <f>IF('Agent 1 Assessment'!C288="","",'Agent 1 Assessment'!C288)</f>
+        <f>IF('Gabrielle Gillie Assessment'!C288="","",'Gabrielle Gillie Assessment'!C288)</f>
         <v/>
       </c>
       <c r="D10" s="11">
@@ -27060,7 +27100,7 @@
       </c>
       <c r="B11" s="34" t="n"/>
       <c r="C11" s="11">
-        <f>IF('Agent 1 Assessment'!C289="","",'Agent 1 Assessment'!C289)</f>
+        <f>IF('Gabrielle Gillie Assessment'!C289="","",'Gabrielle Gillie Assessment'!C289)</f>
         <v/>
       </c>
       <c r="D11" s="11">
@@ -27081,7 +27121,7 @@
         </is>
       </c>
       <c r="K11" s="17">
-        <f>'Agent 1 Assessment'!C3</f>
+        <f>'Gabrielle Gillie Assessment'!C3</f>
         <v/>
       </c>
     </row>
@@ -27093,7 +27133,7 @@
       </c>
       <c r="B12" s="34" t="n"/>
       <c r="C12" s="11">
-        <f>IF('Agent 1 Assessment'!C290="","",'Agent 1 Assessment'!C290*3)</f>
+        <f>IF('Gabrielle Gillie Assessment'!C290="","",'Gabrielle Gillie Assessment'!C290*3)</f>
         <v/>
       </c>
       <c r="D12" s="11">
@@ -33041,7 +33081,7 @@
       </c>
       <c r="B6" s="34" t="n"/>
       <c r="C6" s="12">
-        <f>IF('Agent 2 Assessment'!C285="","",'Agent 2 Assessment'!C285)</f>
+        <f>IF('Dillon Assessment'!C285="","",'Dillon Assessment'!C285)</f>
         <v/>
       </c>
       <c r="D6" s="12">
@@ -33074,7 +33114,7 @@
       </c>
       <c r="B7" s="34" t="n"/>
       <c r="C7" s="12">
-        <f>IF('Agent 2 Assessment'!C284="","",'Agent 2 Assessment'!C284)</f>
+        <f>IF('Dillon Assessment'!C284="","",'Dillon Assessment'!C284)</f>
         <v/>
       </c>
       <c r="D7" s="12">
@@ -33107,7 +33147,7 @@
       </c>
       <c r="B8" s="34" t="n"/>
       <c r="C8" s="11">
-        <f>IF('Agent 2 Assessment'!C286="","",'Agent 2 Assessment'!C286)</f>
+        <f>IF('Dillon Assessment'!C286="","",'Dillon Assessment'!C286)</f>
         <v/>
       </c>
       <c r="D8" s="11">
@@ -33140,7 +33180,7 @@
       </c>
       <c r="B9" s="34" t="n"/>
       <c r="C9" s="11">
-        <f>IF('Agent 2 Assessment'!C287="","",'Agent 2 Assessment'!C287)</f>
+        <f>IF('Dillon Assessment'!C287="","",'Dillon Assessment'!C287)</f>
         <v/>
       </c>
       <c r="D9" s="11">
@@ -33173,7 +33213,7 @@
       </c>
       <c r="B10" s="34" t="n"/>
       <c r="C10" s="11">
-        <f>IF('Agent 2 Assessment'!C288="","",'Agent 2 Assessment'!C288)</f>
+        <f>IF('Dillon Assessment'!C288="","",'Dillon Assessment'!C288)</f>
         <v/>
       </c>
       <c r="D10" s="11">
@@ -33206,7 +33246,7 @@
       </c>
       <c r="B11" s="34" t="n"/>
       <c r="C11" s="11">
-        <f>IF('Agent 2 Assessment'!C289="","",'Agent 2 Assessment'!C289)</f>
+        <f>IF('Dillon Assessment'!C289="","",'Dillon Assessment'!C289)</f>
         <v/>
       </c>
       <c r="D11" s="11">
@@ -33227,7 +33267,7 @@
         </is>
       </c>
       <c r="K11" s="17">
-        <f>'Agent 2 Assessment'!C3</f>
+        <f>'Dillon Assessment'!C3</f>
         <v/>
       </c>
     </row>
@@ -33239,7 +33279,7 @@
       </c>
       <c r="B12" s="34" t="n"/>
       <c r="C12" s="11">
-        <f>IF('Agent 2 Assessment'!C290="","",'Agent 2 Assessment'!C290*3)</f>
+        <f>IF('Dillon Assessment'!C290="","",'Dillon Assessment'!C290*3)</f>
         <v/>
       </c>
       <c r="D12" s="11">
@@ -39187,7 +39227,7 @@
       </c>
       <c r="B6" s="34" t="n"/>
       <c r="C6" s="12">
-        <f>IF('Agent 3 Assessment'!C285="","",'Agent 3 Assessment'!C285)</f>
+        <f>IF('Marcus Lominick Assessment'!C285="","",'Marcus Lominick Assessment'!C285)</f>
         <v/>
       </c>
       <c r="D6" s="12">
@@ -39220,7 +39260,7 @@
       </c>
       <c r="B7" s="34" t="n"/>
       <c r="C7" s="12">
-        <f>IF('Agent 3 Assessment'!C284="","",'Agent 3 Assessment'!C284)</f>
+        <f>IF('Marcus Lominick Assessment'!C284="","",'Marcus Lominick Assessment'!C284)</f>
         <v/>
       </c>
       <c r="D7" s="12">
@@ -39253,7 +39293,7 @@
       </c>
       <c r="B8" s="34" t="n"/>
       <c r="C8" s="11">
-        <f>IF('Agent 3 Assessment'!C286="","",'Agent 3 Assessment'!C286)</f>
+        <f>IF('Marcus Lominick Assessment'!C286="","",'Marcus Lominick Assessment'!C286)</f>
         <v/>
       </c>
       <c r="D8" s="11">
@@ -39286,7 +39326,7 @@
       </c>
       <c r="B9" s="34" t="n"/>
       <c r="C9" s="11">
-        <f>IF('Agent 3 Assessment'!C287="","",'Agent 3 Assessment'!C287)</f>
+        <f>IF('Marcus Lominick Assessment'!C287="","",'Marcus Lominick Assessment'!C287)</f>
         <v/>
       </c>
       <c r="D9" s="11">
@@ -39319,7 +39359,7 @@
       </c>
       <c r="B10" s="34" t="n"/>
       <c r="C10" s="11">
-        <f>IF('Agent 3 Assessment'!C288="","",'Agent 3 Assessment'!C288)</f>
+        <f>IF('Marcus Lominick Assessment'!C288="","",'Marcus Lominick Assessment'!C288)</f>
         <v/>
       </c>
       <c r="D10" s="11">
@@ -39352,7 +39392,7 @@
       </c>
       <c r="B11" s="34" t="n"/>
       <c r="C11" s="11">
-        <f>IF('Agent 3 Assessment'!C289="","",'Agent 3 Assessment'!C289)</f>
+        <f>IF('Marcus Lominick Assessment'!C289="","",'Marcus Lominick Assessment'!C289)</f>
         <v/>
       </c>
       <c r="D11" s="11">
@@ -39373,7 +39413,7 @@
         </is>
       </c>
       <c r="K11" s="17">
-        <f>'Agent 3 Assessment'!C3</f>
+        <f>'Marcus Lominick Assessment'!C3</f>
         <v/>
       </c>
     </row>
@@ -39385,7 +39425,7 @@
       </c>
       <c r="B12" s="34" t="n"/>
       <c r="C12" s="11">
-        <f>IF('Agent 3 Assessment'!C290="","",'Agent 3 Assessment'!C290*3)</f>
+        <f>IF('Marcus Lominick Assessment'!C290="","",'Marcus Lominick Assessment'!C290*3)</f>
         <v/>
       </c>
       <c r="D12" s="11">

</xml_diff>

<commit_message>
Add Nicholas Carnes to score card roster
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hekr7PJ49dGvUHrTGM3jGu
</commit_message>
<xml_diff>
--- a/scorecard/Praedium_Agent_Score_Card.xlsx
+++ b/scorecard/Praedium_Agent_Score_Card.xlsx
@@ -20,8 +20,8 @@
     <sheet name="Mary Elizabeth Young Assessment" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Jayan Abraham Scorecard" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="Jayan Abraham Assessment" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Agent 6 Scorecard" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Agent 6 Assessment" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Nicholas Carnes Scorecard" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Nicholas Carnes Assessment" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="Agent 7 Scorecard" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="Agent 7 Assessment" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
@@ -13363,7 +13363,7 @@
       </c>
       <c r="B6" s="34" t="n"/>
       <c r="C6" s="12">
-        <f>IF('Agent 6 Assessment'!C285="","",'Agent 6 Assessment'!C285)</f>
+        <f>IF('Nicholas Carnes Assessment'!C285="","",'Nicholas Carnes Assessment'!C285)</f>
         <v/>
       </c>
       <c r="D6" s="12">
@@ -13396,7 +13396,7 @@
       </c>
       <c r="B7" s="34" t="n"/>
       <c r="C7" s="12">
-        <f>IF('Agent 6 Assessment'!C284="","",'Agent 6 Assessment'!C284)</f>
+        <f>IF('Nicholas Carnes Assessment'!C284="","",'Nicholas Carnes Assessment'!C284)</f>
         <v/>
       </c>
       <c r="D7" s="12">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="B8" s="34" t="n"/>
       <c r="C8" s="11">
-        <f>IF('Agent 6 Assessment'!C286="","",'Agent 6 Assessment'!C286)</f>
+        <f>IF('Nicholas Carnes Assessment'!C286="","",'Nicholas Carnes Assessment'!C286)</f>
         <v/>
       </c>
       <c r="D8" s="11">
@@ -13462,7 +13462,7 @@
       </c>
       <c r="B9" s="34" t="n"/>
       <c r="C9" s="11">
-        <f>IF('Agent 6 Assessment'!C287="","",'Agent 6 Assessment'!C287)</f>
+        <f>IF('Nicholas Carnes Assessment'!C287="","",'Nicholas Carnes Assessment'!C287)</f>
         <v/>
       </c>
       <c r="D9" s="11">
@@ -13495,7 +13495,7 @@
       </c>
       <c r="B10" s="34" t="n"/>
       <c r="C10" s="11">
-        <f>IF('Agent 6 Assessment'!C288="","",'Agent 6 Assessment'!C288)</f>
+        <f>IF('Nicholas Carnes Assessment'!C288="","",'Nicholas Carnes Assessment'!C288)</f>
         <v/>
       </c>
       <c r="D10" s="11">
@@ -13528,7 +13528,7 @@
       </c>
       <c r="B11" s="34" t="n"/>
       <c r="C11" s="11">
-        <f>IF('Agent 6 Assessment'!C289="","",'Agent 6 Assessment'!C289)</f>
+        <f>IF('Nicholas Carnes Assessment'!C289="","",'Nicholas Carnes Assessment'!C289)</f>
         <v/>
       </c>
       <c r="D11" s="11">
@@ -13549,7 +13549,7 @@
         </is>
       </c>
       <c r="K11" s="17">
-        <f>'Agent 6 Assessment'!C3</f>
+        <f>'Nicholas Carnes Assessment'!C3</f>
         <v/>
       </c>
     </row>
@@ -13561,7 +13561,7 @@
       </c>
       <c r="B12" s="34" t="n"/>
       <c r="C12" s="11">
-        <f>IF('Agent 6 Assessment'!C290="","",'Agent 6 Assessment'!C290*3)</f>
+        <f>IF('Nicholas Carnes Assessment'!C290="","",'Nicholas Carnes Assessment'!C290*3)</f>
         <v/>
       </c>
       <c r="D12" s="11">
@@ -26205,91 +26205,91 @@
         <v/>
       </c>
       <c r="B11" s="17">
-        <f>'Agent 6 Assessment'!C3</f>
+        <f>'Nicholas Carnes Assessment'!C3</f>
         <v/>
       </c>
       <c r="C11" s="18">
-        <f>IFERROR(INDEX('Agent 6 Scorecard'!$Z$15:$Z$80,MATCH($B$3,'Agent 6 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Nicholas Carnes Scorecard'!$Z$15:$Z$80,MATCH($B$3,'Nicholas Carnes Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="D11" s="18">
-        <f>IFERROR(INDEX('Agent 6 Scorecard'!$C$15:$C$80,MATCH($B$3,'Agent 6 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Nicholas Carnes Scorecard'!$C$15:$C$80,MATCH($B$3,'Nicholas Carnes Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="E11" s="18">
-        <f>IFERROR(INDEX('Agent 6 Scorecard'!$E$15:$E$80,MATCH($B$3,'Agent 6 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Nicholas Carnes Scorecard'!$E$15:$E$80,MATCH($B$3,'Nicholas Carnes Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="F11" s="18">
-        <f>IFERROR(INDEX('Agent 6 Scorecard'!$F$15:$F$80,MATCH($B$3,'Agent 6 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Nicholas Carnes Scorecard'!$F$15:$F$80,MATCH($B$3,'Nicholas Carnes Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="G11" s="18">
-        <f>IFERROR(INDEX('Agent 6 Scorecard'!$G$15:$G$80,MATCH($B$3,'Agent 6 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Nicholas Carnes Scorecard'!$G$15:$G$80,MATCH($B$3,'Nicholas Carnes Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="H11" s="18">
-        <f>IFERROR(INDEX('Agent 6 Scorecard'!$H$15:$H$80,MATCH($B$3,'Agent 6 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Nicholas Carnes Scorecard'!$H$15:$H$80,MATCH($B$3,'Nicholas Carnes Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="I11" s="18">
-        <f>IFERROR(INDEX('Agent 6 Scorecard'!$I$15:$I$80,MATCH($B$3,'Agent 6 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Nicholas Carnes Scorecard'!$I$15:$I$80,MATCH($B$3,'Nicholas Carnes Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="J11" s="18">
-        <f>IFERROR(INDEX('Agent 6 Scorecard'!$J$15:$J$80,MATCH($B$3,'Agent 6 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Nicholas Carnes Scorecard'!$J$15:$J$80,MATCH($B$3,'Nicholas Carnes Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="K11" s="18">
-        <f>IFERROR(INDEX('Agent 6 Scorecard'!$K$15:$K$80,MATCH($B$3,'Agent 6 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Nicholas Carnes Scorecard'!$K$15:$K$80,MATCH($B$3,'Nicholas Carnes Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>IFERROR(INDEX('Agent 6 Scorecard'!$L$15:$L$80,MATCH($B$3,'Agent 6 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Nicholas Carnes Scorecard'!$L$15:$L$80,MATCH($B$3,'Nicholas Carnes Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="M11" s="19">
-        <f>'Agent 6 Scorecard'!K10</f>
+        <f>'Nicholas Carnes Scorecard'!K10</f>
         <v/>
       </c>
       <c r="N11" s="19">
-        <f>'Agent 6 Scorecard'!D6</f>
+        <f>'Nicholas Carnes Scorecard'!D6</f>
         <v/>
       </c>
       <c r="O11" s="19">
-        <f>'Agent 6 Scorecard'!C6</f>
+        <f>'Nicholas Carnes Scorecard'!C6</f>
         <v/>
       </c>
       <c r="P11" s="17">
-        <f>'Agent 6 Scorecard'!E6</f>
+        <f>'Nicholas Carnes Scorecard'!E6</f>
         <v/>
       </c>
       <c r="Q11" s="18">
-        <f>'Agent 6 Scorecard'!D8</f>
+        <f>'Nicholas Carnes Scorecard'!D8</f>
         <v/>
       </c>
       <c r="R11" s="18">
-        <f>'Agent 6 Scorecard'!C8</f>
+        <f>'Nicholas Carnes Scorecard'!C8</f>
         <v/>
       </c>
       <c r="S11" s="17">
-        <f>'Agent 6 Scorecard'!K7</f>
+        <f>'Nicholas Carnes Scorecard'!K7</f>
         <v/>
       </c>
       <c r="T11" s="20">
-        <f>'Agent 6 Scorecard'!K8</f>
+        <f>'Nicholas Carnes Scorecard'!K8</f>
         <v/>
       </c>
       <c r="U11" s="21">
-        <f>IF(MAX('Agent 6 Scorecard'!$Y$15:$Y$80)=0,"",MAX('Agent 6 Scorecard'!$Y$15:$Y$80))</f>
+        <f>IF(MAX('Nicholas Carnes Scorecard'!$Y$15:$Y$80)=0,"",MAX('Nicholas Carnes Scorecard'!$Y$15:$Y$80))</f>
         <v/>
       </c>
       <c r="V11" s="22">
-        <f>IFERROR(INDEX('Agent 6 Scorecard'!$V$15:$V$80,MATCH($B$3,'Agent 6 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Nicholas Carnes Scorecard'!$V$15:$V$80,MATCH($B$3,'Nicholas Carnes Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
       <c r="W11" s="22">
-        <f>IFERROR(INDEX('Agent 6 Scorecard'!$W$15:$W$80,MATCH($B$3,'Agent 6 Scorecard'!$A$15:$A$80,0)),"")</f>
+        <f>IFERROR(INDEX('Nicholas Carnes Scorecard'!$W$15:$W$80,MATCH($B$3,'Nicholas Carnes Scorecard'!$A$15:$A$80,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -26760,16 +26760,24 @@
       <c r="A19" s="27" t="n">
         <v>6</v>
       </c>
-      <c r="B19" s="28" t="inlineStr"/>
-      <c r="C19" s="28" t="inlineStr"/>
+      <c r="B19" s="28" t="inlineStr">
+        <is>
+          <t>Nicholas Carnes</t>
+        </is>
+      </c>
+      <c r="C19" s="28" t="inlineStr">
+        <is>
+          <t>ncarnes@kw.com</t>
+        </is>
+      </c>
       <c r="D19" s="29" t="inlineStr">
         <is>
-          <t>Agent 6 Scorecard</t>
+          <t>Nicholas Carnes Scorecard</t>
         </is>
       </c>
       <c r="E19" s="29" t="inlineStr">
         <is>
-          <t>Agent 6 Assessment</t>
+          <t>Nicholas Carnes Assessment</t>
         </is>
       </c>
       <c r="F19" s="28" t="inlineStr"/>

</xml_diff>